<commit_message>
fix: remove orphaned Mappings tab button and fix card heights in System Settings
</commit_message>
<xml_diff>
--- a/Scholarships.xlsx
+++ b/Scholarships.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\NU\Nile_ERP\Finance---A-R\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{870C5D40-B4F2-4877-AD31-8033EF654016}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{751B9CAD-C814-4282-9BD3-96C5D38F419D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15645" xr2:uid="{15FD632E-8033-48B4-8775-86E97D9C9AB5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="40">
   <si>
     <t>Charge code</t>
   </si>
@@ -156,6 +156,9 @@
   </si>
   <si>
     <t>SC.Rass.PG</t>
+  </si>
+  <si>
+    <t>Category</t>
   </si>
 </sst>
 </file>
@@ -547,6 +550,9 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
+      <c r="B1" s="1" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">

</xml_diff>